<commit_message>
add and move data
</commit_message>
<xml_diff>
--- a/data-raw/data/vanwiechen_percentage_cm.xlsx
+++ b/data-raw/data/vanwiechen_percentage_cm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eekhouti\Documents\GitHub\dscoreddi\data-raw\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365tno-my.sharepoint.com/personal/iris_eekhout_tno_nl/Documents/Documents/GitHub/dscoreddi/data-raw/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B30940C-EB09-4A6A-8809-3723A2EFB270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{6B30940C-EB09-4A6A-8809-3723A2EFB270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC45EE80-7DAF-4D6F-A7DA-14F8A7D5A655}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3A27370D-2517-4338-AE96-3179580301A2}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3A27370D-2517-4338-AE96-3179580301A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -1466,12 +1466,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B7702C6-8B19-495E-897D-E69691612534}">
   <dimension ref="A1:J122"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="5" width="9.140625" style="17"/>
+    <col min="1" max="3" width="19" customWidth="1"/>
+    <col min="4" max="5" width="19" style="17" customWidth="1"/>
+    <col min="6" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="115.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="117.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1503,7 +1505,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1511,7 +1513,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="6">
-        <v>44654</v>
+        <v>45750</v>
       </c>
       <c r="D2" s="13">
         <v>3</v>
@@ -1533,7 +1535,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3">
         <f>A2</f>
         <v>1</v>
@@ -1565,7 +1567,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3">
         <v>29</v>
       </c>
@@ -1597,7 +1599,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3">
         <f>A4</f>
         <v>29</v>
@@ -1631,7 +1633,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3">
         <v>52</v>
       </c>
@@ -1661,7 +1663,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="10">
         <f t="shared" ref="A7" si="0">A6</f>
         <v>52</v>
@@ -1692,7 +1694,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="10">
         <v>53</v>
       </c>
@@ -1722,7 +1724,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10">
         <v>53</v>
       </c>
@@ -1752,7 +1754,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>56</v>
       </c>
@@ -1782,7 +1784,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="3">
         <f>A10</f>
         <v>56</v>
@@ -1814,7 +1816,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -1846,7 +1848,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3">
         <f>A12</f>
         <v>2</v>
@@ -1880,7 +1882,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3">
         <v>2</v>
       </c>
@@ -1912,7 +1914,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3">
         <f>A14</f>
         <v>2</v>
@@ -1944,7 +1946,7 @@
       </c>
       <c r="J15" s="4"/>
     </row>
-    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>30</v>
       </c>
@@ -1976,7 +1978,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="3">
         <f>A16</f>
         <v>30</v>
@@ -2010,7 +2012,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="3">
         <v>3</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="3">
         <f>A18</f>
         <v>3</v>
@@ -2070,7 +2072,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="3">
         <v>3</v>
       </c>
@@ -2098,7 +2100,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="3">
         <f>A20</f>
         <v>3</v>
@@ -2128,7 +2130,7 @@
       <c r="I21" s="8"/>
       <c r="J21" s="8"/>
     </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="3">
         <v>4</v>
       </c>
@@ -2156,7 +2158,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="3">
         <f>A22</f>
         <v>4</v>
@@ -2190,7 +2192,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="3">
         <v>31</v>
       </c>
@@ -2218,7 +2220,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="3">
         <f>A24</f>
         <v>31</v>
@@ -2252,7 +2254,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="3">
         <v>54</v>
       </c>
@@ -2280,7 +2282,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="3">
         <f>A26</f>
         <v>54</v>
@@ -2312,7 +2314,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="3">
         <v>57</v>
       </c>
@@ -2338,7 +2340,7 @@
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
     </row>
-    <row r="29" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="3">
         <f>A28</f>
         <v>57</v>
@@ -2370,7 +2372,7 @@
       </c>
       <c r="J29" s="4"/>
     </row>
-    <row r="30" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="3">
         <v>5</v>
       </c>
@@ -2398,7 +2400,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="3">
         <f>A30</f>
         <v>5</v>
@@ -2432,7 +2434,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="3">
         <v>6</v>
       </c>
@@ -2460,7 +2462,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="3">
         <f>A32</f>
         <v>6</v>
@@ -2494,7 +2496,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="3">
         <v>6</v>
       </c>
@@ -2522,7 +2524,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="3">
         <f>A34</f>
         <v>6</v>
@@ -2554,7 +2556,7 @@
       </c>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="3">
         <v>32</v>
       </c>
@@ -2580,7 +2582,7 @@
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
     </row>
-    <row r="37" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="3">
         <f>A36</f>
         <v>32</v>
@@ -2608,7 +2610,7 @@
       <c r="I37" s="4"/>
       <c r="J37" s="4"/>
     </row>
-    <row r="38" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="3">
         <v>55</v>
       </c>
@@ -2636,7 +2638,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="3">
         <f>A38</f>
         <v>55</v>
@@ -2670,7 +2672,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="3">
         <v>58</v>
       </c>
@@ -2696,7 +2698,7 @@
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
     </row>
-    <row r="41" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="3">
         <f>A40</f>
         <v>58</v>
@@ -2728,7 +2730,7 @@
       </c>
       <c r="J41" s="4"/>
     </row>
-    <row r="42" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="3">
         <v>59</v>
       </c>
@@ -2758,7 +2760,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="3">
         <v>59</v>
       </c>
@@ -2788,7 +2790,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="3">
         <v>7</v>
       </c>
@@ -2816,7 +2818,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="3">
         <f>A44</f>
         <v>7</v>
@@ -2850,7 +2852,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="3">
         <v>8</v>
       </c>
@@ -2878,7 +2880,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="3">
         <f>A46</f>
         <v>8</v>
@@ -2912,7 +2914,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="3">
         <v>9</v>
       </c>
@@ -2940,7 +2942,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="3">
         <f>A48</f>
         <v>9</v>
@@ -2972,7 +2974,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="3">
         <v>9</v>
       </c>
@@ -3000,7 +3002,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="3">
         <f>A50</f>
         <v>9</v>
@@ -3030,7 +3032,7 @@
       <c r="I51" s="4"/>
       <c r="J51" s="4"/>
     </row>
-    <row r="52" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="3">
         <v>33</v>
       </c>
@@ -3058,7 +3060,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="3">
         <f>A52</f>
         <v>33</v>
@@ -3092,7 +3094,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="3">
         <v>60</v>
       </c>
@@ -3120,7 +3122,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="3">
         <f>A54</f>
         <v>60</v>
@@ -3154,7 +3156,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="3">
         <v>61</v>
       </c>
@@ -3182,7 +3184,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="3">
         <f>A56</f>
         <v>61</v>
@@ -3216,7 +3218,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="3">
         <v>62</v>
       </c>
@@ -3246,7 +3248,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="3">
         <v>10</v>
       </c>
@@ -3274,7 +3276,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="3">
         <f>A59</f>
         <v>10</v>
@@ -3308,7 +3310,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="3">
         <v>10</v>
       </c>
@@ -3336,7 +3338,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="3">
         <f>A61</f>
         <v>10</v>
@@ -3368,7 +3370,7 @@
       </c>
       <c r="J62" s="4"/>
     </row>
-    <row r="63" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="3">
         <v>34</v>
       </c>
@@ -3396,7 +3398,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="3">
         <f>A63</f>
         <v>34</v>
@@ -3430,7 +3432,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="3">
         <v>35</v>
       </c>
@@ -3458,7 +3460,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="3">
         <f>A65</f>
         <v>35</v>
@@ -3488,7 +3490,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="3">
         <v>36</v>
       </c>
@@ -3516,7 +3518,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="3">
         <f>A67</f>
         <v>36</v>
@@ -3550,7 +3552,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="3">
         <v>63</v>
       </c>
@@ -3578,7 +3580,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="3">
         <f>A69</f>
         <v>63</v>
@@ -3612,7 +3614,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="3">
         <v>64</v>
       </c>
@@ -3640,7 +3642,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="3">
         <f>A71</f>
         <v>64</v>
@@ -3674,7 +3676,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="3">
         <v>65</v>
       </c>
@@ -3702,7 +3704,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="3">
         <f>A73</f>
         <v>65</v>
@@ -3736,7 +3738,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="3">
         <v>11</v>
       </c>
@@ -3764,7 +3766,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="3">
         <f>A75</f>
         <v>11</v>
@@ -3796,7 +3798,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="3">
         <v>11</v>
       </c>
@@ -3824,7 +3826,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="3">
         <f>A77</f>
         <v>11</v>
@@ -3854,7 +3856,7 @@
       <c r="I78" s="8"/>
       <c r="J78" s="8"/>
     </row>
-    <row r="79" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="3">
         <v>12</v>
       </c>
@@ -3882,7 +3884,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="3">
         <f>A79</f>
         <v>12</v>
@@ -3916,7 +3918,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="3">
         <v>37</v>
       </c>
@@ -3944,7 +3946,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="3">
         <f t="shared" ref="A82:A84" si="1">A81</f>
         <v>37</v>
@@ -3978,7 +3980,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="3">
         <f t="shared" si="1"/>
         <v>37</v>
@@ -4012,7 +4014,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="3">
         <f t="shared" si="1"/>
         <v>37</v>
@@ -4046,7 +4048,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="3">
         <v>38</v>
       </c>
@@ -4072,7 +4074,7 @@
       <c r="I85" s="4"/>
       <c r="J85" s="4"/>
     </row>
-    <row r="86" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="3">
         <f>A85</f>
         <v>38</v>
@@ -4104,7 +4106,7 @@
       </c>
       <c r="J86" s="4"/>
     </row>
-    <row r="87" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="3">
         <v>66</v>
       </c>
@@ -4132,7 +4134,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="3">
         <f>A87</f>
         <v>66</v>
@@ -4166,7 +4168,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="3">
         <v>67</v>
       </c>
@@ -4194,7 +4196,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="3">
         <f>A89</f>
         <v>67</v>
@@ -4228,7 +4230,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="3">
         <v>13</v>
       </c>
@@ -4260,7 +4262,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="3">
         <f>A91</f>
         <v>13</v>
@@ -4294,7 +4296,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="3">
         <v>13</v>
       </c>
@@ -4326,7 +4328,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="3">
         <f>A93</f>
         <v>13</v>
@@ -4358,7 +4360,7 @@
       </c>
       <c r="J94" s="4"/>
     </row>
-    <row r="95" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="3">
         <v>14</v>
       </c>
@@ -4388,7 +4390,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="3">
         <f>A95</f>
         <v>14</v>
@@ -4420,7 +4422,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="3">
         <v>39</v>
       </c>
@@ -4452,7 +4454,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="3">
         <f>A97</f>
         <v>39</v>
@@ -4486,7 +4488,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="3">
         <v>40</v>
       </c>
@@ -4514,7 +4516,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="3">
         <f>A99</f>
         <v>40</v>
@@ -4544,7 +4546,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="3">
         <v>68</v>
       </c>
@@ -4576,7 +4578,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="3">
         <f>A101</f>
         <v>68</v>
@@ -4610,7 +4612,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="3">
         <v>69</v>
       </c>
@@ -4638,7 +4640,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="3">
         <f>A103</f>
         <v>69</v>
@@ -4668,7 +4670,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="3">
         <v>15</v>
       </c>
@@ -4692,7 +4694,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="3">
         <f>A105</f>
         <v>15</v>
@@ -4722,7 +4724,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="3">
         <v>15</v>
       </c>
@@ -4746,7 +4748,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="3">
         <f>A107</f>
         <v>15</v>
@@ -4774,7 +4776,7 @@
       </c>
       <c r="J108" s="4"/>
     </row>
-    <row r="109" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="3">
         <v>16</v>
       </c>
@@ -4798,7 +4800,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="3">
         <f>A109</f>
         <v>16</v>
@@ -4828,7 +4830,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="111" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="3">
         <v>41</v>
       </c>
@@ -4852,7 +4854,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="3">
         <f t="shared" ref="A112:A115" si="3">A111</f>
         <v>41</v>
@@ -4882,7 +4884,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="113" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="3">
         <f t="shared" si="3"/>
         <v>41</v>
@@ -4912,7 +4914,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="3">
         <f t="shared" si="3"/>
         <v>41</v>
@@ -4942,7 +4944,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="3">
         <f t="shared" si="3"/>
         <v>41</v>
@@ -4972,7 +4974,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="3">
         <v>42</v>
       </c>
@@ -4994,7 +4996,7 @@
       <c r="I116" s="4"/>
       <c r="J116" s="4"/>
     </row>
-    <row r="117" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="3">
         <f t="shared" ref="A117:A118" si="5">A116</f>
         <v>42</v>
@@ -5018,7 +5020,7 @@
       <c r="I117" s="4"/>
       <c r="J117" s="4"/>
     </row>
-    <row r="118" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="3">
         <f t="shared" si="5"/>
         <v>42</v>
@@ -5042,7 +5044,7 @@
       <c r="I118" s="4"/>
       <c r="J118" s="4"/>
     </row>
-    <row r="119" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="3">
         <v>68</v>
       </c>
@@ -5066,7 +5068,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="3">
         <f>A119</f>
         <v>68</v>
@@ -5094,7 +5096,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="3">
         <v>70</v>
       </c>
@@ -5118,7 +5120,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A122" s="3">
         <f>A121</f>
         <v>70</v>

</xml_diff>

<commit_message>
update paper results - submission 13-3-2025
</commit_message>
<xml_diff>
--- a/data-raw/data/vanwiechen_percentage_cm.xlsx
+++ b/data-raw/data/vanwiechen_percentage_cm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365tno-my.sharepoint.com/personal/iris_eekhout_tno_nl/Documents/Documents/GitHub/dscoreddi/data-raw/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{6B30940C-EB09-4A6A-8809-3723A2EFB270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC45EE80-7DAF-4D6F-A7DA-14F8A7D5A655}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{6B30940C-EB09-4A6A-8809-3723A2EFB270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEAFD9AB-0145-4F9F-AA63-A150CEB69E0C}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3A27370D-2517-4338-AE96-3179580301A2}"/>
+    <workbookView xWindow="57765" yWindow="0" windowWidth="22740" windowHeight="20985" xr2:uid="{3A27370D-2517-4338-AE96-3179580301A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="331">
   <si>
     <t>Kenmerk</t>
   </si>
@@ -954,12 +954,120 @@
   <si>
     <t>week2</t>
   </si>
+  <si>
+    <t>bouwt vrachtauto na</t>
+  </si>
+  <si>
+    <t>  524/628</t>
+  </si>
+  <si>
+    <t>5.055/5.957</t>
+  </si>
+  <si>
+    <t>2.600/3.009</t>
+  </si>
+  <si>
+    <t>1.163/1.290</t>
+  </si>
+  <si>
+    <t>plaatst 3 vormen in stoof</t>
+  </si>
+  <si>
+    <t>  623/660</t>
+  </si>
+  <si>
+    <t>4833/6153</t>
+  </si>
+  <si>
+    <t>tekent verticale lijn na</t>
+  </si>
+  <si>
+    <t>  538/584</t>
+  </si>
+  <si>
+    <t>5.152/5.543</t>
+  </si>
+  <si>
+    <t>zegt ‘zinnen’ van 3 of meer woorden</t>
+  </si>
+  <si>
+    <t>  654/686</t>
+  </si>
+  <si>
+    <t>6.161/6.430</t>
+  </si>
+  <si>
+    <t>is verstaanbaar voor bekenden</t>
+  </si>
+  <si>
+    <t>  633/665</t>
+  </si>
+  <si>
+    <t>5.985/6.253</t>
+  </si>
+  <si>
+    <t>loopt soepel</t>
+  </si>
+  <si>
+    <t>  643/643</t>
+  </si>
+  <si>
+    <t>6.171/6.175</t>
+  </si>
+  <si>
+    <t>fietst (op driewieler)</t>
+  </si>
+  <si>
+    <t>  449/550</t>
+  </si>
+  <si>
+    <t>4.421/5.151</t>
+  </si>
+  <si>
+    <t>2.197/2.542</t>
+  </si>
+  <si>
+    <t>  988/1.095</t>
+  </si>
+  <si>
+    <t>1.175/1.214</t>
+  </si>
+  <si>
+    <t>tekent cirkel na</t>
+  </si>
+  <si>
+    <t>1.974/2.120</t>
+  </si>
+  <si>
+    <t>2.150/2.280</t>
+  </si>
+  <si>
+    <t>is goed verstaanbaar voor onderzoeker</t>
+  </si>
+  <si>
+    <t>1.725/1.977</t>
+  </si>
+  <si>
+    <t>1.892/2.123</t>
+  </si>
+  <si>
+    <t>1.501/1.640</t>
+  </si>
+  <si>
+    <t>stelt vragen naar ‘hoeveel’, ‘wanneer’, ‘waarom’</t>
+  </si>
+  <si>
+    <t>1.838/1.914</t>
+  </si>
+  <si>
+    <t>2.013/2.068</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -997,8 +1105,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF222222"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1011,8 +1131,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1094,12 +1220,141 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFDADADA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD5D5D5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFD5D5D5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFD5D5D5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFDADADA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD5D5D5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD5D5D5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFDADADA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD5D5D5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD5D5D5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD5D5D5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD5D5D5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD5D5D5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD5D5D5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFD5D5D5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFDADADA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1150,6 +1405,55 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1168,10 +1472,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1209,7 +1517,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1315,7 +1623,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1457,7 +1765,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1465,7 +1773,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B7702C6-8B19-495E-897D-E69691612534}">
-  <dimension ref="A1:J122"/>
+  <dimension ref="A1:J148"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="19" customWidth="1"/>
@@ -5150,7 +5458,409 @@
         <v>292</v>
       </c>
     </row>
+    <row r="123" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A123" s="22">
+        <v>20</v>
+      </c>
+      <c r="B123" s="22" t="s">
+        <v>295</v>
+      </c>
+      <c r="C123" s="20">
+        <v>35</v>
+      </c>
+      <c r="F123" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="G123" s="20">
+        <v>83.4</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A124" s="23"/>
+      <c r="B124" s="23"/>
+      <c r="C124" s="19">
+        <v>36</v>
+      </c>
+      <c r="F124" s="19" t="s">
+        <v>297</v>
+      </c>
+      <c r="G124" s="19">
+        <v>84.9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A125" s="23"/>
+      <c r="B125" s="23"/>
+      <c r="C125" s="19">
+        <v>37</v>
+      </c>
+      <c r="F125" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="G125" s="19">
+        <v>86.4</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A126" s="24"/>
+      <c r="B126" s="24"/>
+      <c r="C126" s="19">
+        <v>38</v>
+      </c>
+      <c r="F126" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="G126" s="19">
+        <v>90.2</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A127" s="25">
+        <v>21</v>
+      </c>
+      <c r="B127" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="C127" s="19">
+        <v>35</v>
+      </c>
+      <c r="F127" s="19" t="s">
+        <v>301</v>
+      </c>
+      <c r="G127" s="19">
+        <v>94.4</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A128" s="26"/>
+      <c r="B128" s="26"/>
+      <c r="C128" s="21">
+        <v>36</v>
+      </c>
+      <c r="D128" s="21"/>
+      <c r="E128" s="21"/>
+      <c r="F128" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="G128">
+        <v>94.8</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A129" s="30">
+        <v>22</v>
+      </c>
+      <c r="B129" s="30" t="s">
+        <v>303</v>
+      </c>
+      <c r="C129" s="28">
+        <v>35</v>
+      </c>
+      <c r="F129" s="28" t="s">
+        <v>304</v>
+      </c>
+      <c r="G129" s="28">
+        <v>92.1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A130" s="31"/>
+      <c r="B130" s="31"/>
+      <c r="C130" s="27">
+        <v>36</v>
+      </c>
+      <c r="F130" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="G130" s="27">
+        <v>92.9</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A131" s="33">
+        <v>45</v>
+      </c>
+      <c r="B131" s="33" t="s">
+        <v>306</v>
+      </c>
+      <c r="C131" s="27">
+        <v>35</v>
+      </c>
+      <c r="F131" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="G131" s="27">
+        <v>95.3</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A132" s="31"/>
+      <c r="B132" s="31"/>
+      <c r="C132" s="27">
+        <v>36</v>
+      </c>
+      <c r="F132" s="27" t="s">
+        <v>308</v>
+      </c>
+      <c r="G132" s="27">
+        <v>95.8</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A133" s="33">
+        <v>46</v>
+      </c>
+      <c r="B133" s="33" t="s">
+        <v>309</v>
+      </c>
+      <c r="C133" s="27">
+        <v>35</v>
+      </c>
+      <c r="F133" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="G133" s="27">
+        <v>95.2</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A134" s="31"/>
+      <c r="B134" s="31"/>
+      <c r="C134" s="27">
+        <v>36</v>
+      </c>
+      <c r="F134" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="G134" s="27">
+        <v>95.7</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A135" s="33">
+        <v>68</v>
+      </c>
+      <c r="B135" s="33" t="s">
+        <v>312</v>
+      </c>
+      <c r="C135" s="27">
+        <v>35</v>
+      </c>
+      <c r="F135" s="27" t="s">
+        <v>313</v>
+      </c>
+      <c r="G135" s="27">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A136" s="31"/>
+      <c r="B136" s="31"/>
+      <c r="C136" s="27">
+        <v>36</v>
+      </c>
+      <c r="F136" s="27" t="s">
+        <v>314</v>
+      </c>
+      <c r="G136" s="27">
+        <v>99.9</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A137" s="33">
+        <v>73</v>
+      </c>
+      <c r="B137" s="33" t="s">
+        <v>315</v>
+      </c>
+      <c r="C137" s="27">
+        <v>35</v>
+      </c>
+      <c r="F137" s="27" t="s">
+        <v>316</v>
+      </c>
+      <c r="G137" s="27">
+        <v>81.599999999999994</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A138" s="32"/>
+      <c r="B138" s="32"/>
+      <c r="C138" s="27">
+        <v>36</v>
+      </c>
+      <c r="F138" s="27" t="s">
+        <v>317</v>
+      </c>
+      <c r="G138" s="27">
+        <v>85.8</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A139" s="32"/>
+      <c r="B139" s="32"/>
+      <c r="C139" s="27">
+        <v>37</v>
+      </c>
+      <c r="F139" s="27" t="s">
+        <v>318</v>
+      </c>
+      <c r="G139" s="27">
+        <v>86.4</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A140" s="32"/>
+      <c r="B140" s="32"/>
+      <c r="C140" s="27">
+        <v>38</v>
+      </c>
+      <c r="F140" s="27" t="s">
+        <v>319</v>
+      </c>
+      <c r="G140" s="27">
+        <v>90.2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A141" s="31"/>
+      <c r="B141" s="31"/>
+      <c r="C141" s="27">
+        <v>45</v>
+      </c>
+      <c r="F141" s="27" t="s">
+        <v>320</v>
+      </c>
+      <c r="G141" s="27">
+        <v>96.8</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A142" s="33">
+        <v>26</v>
+      </c>
+      <c r="B142" s="33" t="s">
+        <v>321</v>
+      </c>
+      <c r="C142" s="27">
+        <v>46</v>
+      </c>
+      <c r="F142" s="27" t="s">
+        <v>322</v>
+      </c>
+      <c r="G142" s="27">
+        <v>93.1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A143" s="31"/>
+      <c r="B143" s="31"/>
+      <c r="C143" s="27">
+        <v>47</v>
+      </c>
+      <c r="F143" s="27" t="s">
+        <v>323</v>
+      </c>
+      <c r="G143" s="27">
+        <v>94.3</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A144" s="33">
+        <v>49</v>
+      </c>
+      <c r="B144" s="33" t="s">
+        <v>324</v>
+      </c>
+      <c r="C144" s="27">
+        <v>46</v>
+      </c>
+      <c r="F144" s="27" t="s">
+        <v>325</v>
+      </c>
+      <c r="G144" s="27">
+        <v>87.3</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A145" s="32"/>
+      <c r="B145" s="32"/>
+      <c r="C145" s="27">
+        <v>47</v>
+      </c>
+      <c r="F145" s="27" t="s">
+        <v>326</v>
+      </c>
+      <c r="G145" s="27">
+        <v>98.1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A146" s="31"/>
+      <c r="B146" s="31"/>
+      <c r="C146" s="27">
+        <v>48</v>
+      </c>
+      <c r="F146" s="27" t="s">
+        <v>327</v>
+      </c>
+      <c r="G146" s="27">
+        <v>91.5</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" ht="23.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A147" s="33">
+        <v>50</v>
+      </c>
+      <c r="B147" s="33" t="s">
+        <v>328</v>
+      </c>
+      <c r="C147" s="27">
+        <v>46</v>
+      </c>
+      <c r="F147" s="27" t="s">
+        <v>329</v>
+      </c>
+      <c r="G147" s="27">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A148" s="34"/>
+      <c r="B148" s="34"/>
+      <c r="C148" s="29">
+        <v>47</v>
+      </c>
+      <c r="F148" s="29" t="s">
+        <v>330</v>
+      </c>
+      <c r="G148" s="29">
+        <v>97.3</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="A147:A148"/>
+    <mergeCell ref="B147:B148"/>
+    <mergeCell ref="A142:A143"/>
+    <mergeCell ref="B142:B143"/>
+    <mergeCell ref="A144:A146"/>
+    <mergeCell ref="B144:B146"/>
+    <mergeCell ref="A135:A136"/>
+    <mergeCell ref="B135:B136"/>
+    <mergeCell ref="A137:A141"/>
+    <mergeCell ref="B137:B141"/>
+    <mergeCell ref="A131:A132"/>
+    <mergeCell ref="B131:B132"/>
+    <mergeCell ref="A133:A134"/>
+    <mergeCell ref="B133:B134"/>
+    <mergeCell ref="A129:A130"/>
+    <mergeCell ref="B129:B130"/>
+    <mergeCell ref="A123:A126"/>
+    <mergeCell ref="B123:B126"/>
+    <mergeCell ref="A127:A128"/>
+    <mergeCell ref="B127:B128"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="https://www.ncj.nl/van-wiechen/kenmerken/details/?item=1" xr:uid="{B48A6452-8512-44FE-BD35-91A7075898B4}"/>
     <hyperlink ref="B4" r:id="rId2" display="https://www.ncj.nl/van-wiechen/kenmerken/details/?item=29" xr:uid="{8CC66355-703D-4DCF-9E32-5300CD9CE740}"/>

</xml_diff>